<commit_message>
agregue dos modelos uno fileDrive y otro folderDrive
</commit_message>
<xml_diff>
--- a/LISTAS/ma/SOPORTE LATERAL TUBULAR DISMAY.xlsx
+++ b/LISTAS/ma/SOPORTE LATERAL TUBULAR DISMAY.xlsx
@@ -918,14 +918,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="18" t="n">
-        <v>45163.60925258535</v>
+        <v>45218</v>
       </c>
       <c r="E1" s="7" t="n"/>
     </row>
-    <row r="2"/>
-    <row r="3"/>
-    <row r="4"/>
-    <row r="5"/>
     <row r="6" ht="22.5" customHeight="1" s="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
@@ -971,15 +967,7 @@
       </c>
       <c r="E11" s="12" t="n"/>
     </row>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
     <row r="19" hidden="1" s="1"/>
-    <row r="20"/>
     <row r="21" ht="18" customHeight="1" s="1">
       <c r="A21" s="24" t="inlineStr">
         <is>
@@ -1011,7 +999,7 @@
       </c>
       <c r="C22" s="32" t="n"/>
       <c r="D22" s="33" t="n">
-        <v>329.033</v>
+        <v>361.9363</v>
       </c>
     </row>
     <row r="23" ht="19.5" customHeight="1" s="1">
@@ -1030,13 +1018,6 @@
         <v>416.963</v>
       </c>
     </row>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
     <row r="31" ht="12" customHeight="1" s="1"/>
     <row r="32" hidden="1" ht="18" customHeight="1" s="1">
       <c r="E32" s="4" t="n"/>
@@ -1104,12 +1085,8 @@
     <row r="37" ht="18" customHeight="1" s="1">
       <c r="E37" s="4" t="n"/>
     </row>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
     <row r="41" ht="6.75" customHeight="1" s="1"/>
     <row r="42" hidden="1" s="1"/>
-    <row r="43"/>
     <row r="44" ht="18" customHeight="1" s="1">
       <c r="A44" s="24" t="inlineStr">
         <is>
@@ -1160,7 +1137,6 @@
         <v>446.745</v>
       </c>
     </row>
-    <row r="47"/>
     <row r="48" ht="15" customHeight="1" s="1">
       <c r="A48" s="28" t="inlineStr">
         <is>
@@ -1168,8 +1144,6 @@
         </is>
       </c>
     </row>
-    <row r="49"/>
-    <row r="50"/>
     <row r="51" ht="15.75" customHeight="1" s="1">
       <c r="A51" s="5" t="n"/>
     </row>
@@ -1178,20 +1152,20 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="A48:D48"/>
+    <mergeCell ref="B34:C34"/>
     <mergeCell ref="B45:C45"/>
     <mergeCell ref="B46:C46"/>
     <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="A48:D48"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A10:D10"/>
     <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="A9:D9"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A11:D11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>